<commit_message>
YA ESTA COMPLETO REVISAT CON LA FIRMAEC
</commit_message>
<xml_diff>
--- a/app/static/temp/Base_Tramites_INAMHI.xlsx
+++ b/app/static/temp/Base_Tramites_INAMHI.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -474,7 +474,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>#30</t>
+          <t>#31</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -499,34 +499,34 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>27/07/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>#29</t>
+          <t>#30</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1723929162</t>
+          <t>9999999999</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ALEXIS  AMAGUA</t>
+          <t xml:space="preserve">MARIO ORLANDO GOMEZ JACOME </t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>alejo@gmail.com</t>
+          <t>9999999999@inamhi.gob.ec</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CREADO</t>
+          <t>NEGADO</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -538,54 +538,54 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>#27</t>
+          <t>#29</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1723929160</t>
+          <t>1723929162</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>OLIVER MARTINEZ</t>
+          <t>ALEXIS  AMAGUA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>alex@gmail.com</t>
+          <t>alejo@gmail.com</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CREADO</t>
+          <t>APROBADO</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>27/07/2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>#24</t>
+          <t>#27</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0102484342</t>
+          <t>1723929160</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DAMARIS TAYO</t>
+          <t>OLIVER MARTINEZ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>dtayo@inamhi.ec</t>
+          <t>alex@gmail.com</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -595,29 +595,29 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>23/07/2026</t>
+          <t>24/07/2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>#23</t>
+          <t>#24</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1723929192</t>
+          <t>0102484342</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>VERO REINO</t>
+          <t>DAMARIS TAYO</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>vreino@inamhi.gob.ec</t>
+          <t>dtayo@inamhi.ec</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -627,37 +627,69 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>22/07/2026</t>
+          <t>23/07/2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>#23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1723929192</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>VERO REINO</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>vreino@inamhi.gob.ec</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>22/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>#22</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>1752459854</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t xml:space="preserve">JOSTIN SALAZAR </t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>jsalazar@inamhi.gob.ec</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>CREADO</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>22/07/2026</t>
         </is>

</xml_diff>